<commit_message>
Migrate to welogx.com domain and update GA4 tracking
- Update GA4 tracking ID to G-HFZWKT7TVE
- Migrate all URLs from ewltl.com to welogx.com
- Update Cognito callback URLs
- Remove hardcoded secrets from route files (use env vars)
- Add deploy scripts to .gitignore for security
- Delete old task definition JSON files

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/BOL-TEMPLATE .xlsx
+++ b/BOL-TEMPLATE .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ftlfb\Desktop\Shipments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ew-josh/Downloads/EW-Design/EW-WebView/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4520923C-8EF1-4973-AAE2-011CEF383DB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5FF4010-C824-5C43-868C-C6C225398B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{B7742BF1-83A5-4DA7-805C-D71377E9CF30}"/>
+    <workbookView xWindow="39860" yWindow="-4380" windowWidth="25820" windowHeight="15500" xr2:uid="{B7742BF1-83A5-4DA7-805C-D71377E9CF30}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Page</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>Customer Order No.</t>
-  </si>
-  <si>
-    <t># of Packages</t>
   </si>
   <si>
     <t>Weight</t>
@@ -302,49 +299,6 @@
     <t>SHIPMENT INFORMATION</t>
   </si>
   <si>
-    <t>Handling Unit</t>
-  </si>
-  <si>
-    <t>Qty</t>
-  </si>
-  <si>
-    <t>Handling Type</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Commodity Description</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Commodities requiring special or additional care or attention in handling or stowing must be so marked and packaged as to ensure safe transportation with ordinary care. See Section 2(e) of NMFC item 360</t>
-    </r>
-  </si>
-  <si>
     <t>Where the rate is dependent on value, shippers are required to state specifically in writing the agreed or declared value of the property as follows: “The agreed or declared value of the property is specifically stated by the shipper to be not exceeding _______________ per _______________.</t>
   </si>
   <si>
@@ -521,13 +475,32 @@
       <t>_______________________________________________
 Carrier acknowledges receipt of packages and required placards. Carrier certifies emergency response information was made available and/or carrier has the DOT emergency response guidebook or equivalent documentation in the vehicle. Property described above is received in good order, except as noted.</t>
     </r>
+  </si>
+  <si>
+    <t>Pallet</t>
+  </si>
+  <si>
+    <t>Pieces</t>
+  </si>
+  <si>
+    <t># of Pallets</t>
+  </si>
+  <si>
+    <t>Total Weight</t>
+  </si>
+  <si>
+    <t>Commodity Description
+Commodities requiring special or additional care or attention in handling or stowing must be so marked and packaged as to ensure safe transportation with ordinary care. See Section 2(e) of NMFC item 360</t>
+  </si>
+  <si>
+    <t>Class</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -597,6 +570,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -612,7 +598,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -715,12 +701,99 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -731,53 +804,25 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -787,42 +832,65 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1176,492 +1244,491 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C2565DD-4DEC-4CF1-9315-F68EDF44971F}">
   <dimension ref="A1:I34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.54296875" customWidth="1"/>
-    <col min="2" max="2" width="9.90625" customWidth="1"/>
-    <col min="3" max="3" width="6.6328125" customWidth="1"/>
-    <col min="4" max="4" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="6.5" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
+    <col min="3" max="3" width="13.5" customWidth="1"/>
+    <col min="4" max="4" width="12.5" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="9.36328125" customWidth="1"/>
-    <col min="7" max="7" width="11.7265625" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" customWidth="1"/>
     <col min="8" max="8" width="1" customWidth="1"/>
-    <col min="9" max="9" width="20.1796875" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+    </row>
+    <row r="3" spans="1:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="30" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-    </row>
-    <row r="3" spans="1:9" ht="59" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9" t="s">
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+    </row>
+    <row r="5" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-    </row>
-    <row r="5" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="9" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-    </row>
-    <row r="7" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="20" t="s">
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+    </row>
+    <row r="7" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="20" t="s">
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="22" t="s">
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="24"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="20"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="25" t="s">
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="25"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G9" s="26" t="s">
         <v>10</v>
       </c>
       <c r="H9" s="26"/>
-      <c r="I9" s="27" t="s">
+      <c r="I9" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="28" t="b">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="G10" s="21" t="b">
+      <c r="G10" s="27" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="21"/>
-      <c r="I10" s="29" t="b">
+      <c r="H10" s="27"/>
+      <c r="I10" s="6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10" t="s">
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="28"/>
+      <c r="H12" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="21"/>
+    </row>
+    <row r="13" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="21"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="29"/>
+    </row>
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I12" s="9"/>
-    </row>
-    <row r="13" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+      <c r="D16" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="35"/>
+      <c r="F16" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="H16" s="31"/>
+      <c r="I16" s="32"/>
+    </row>
+    <row r="17" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="10"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="42"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="41"/>
+      <c r="I19" s="42"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-    </row>
-    <row r="17" spans="1:9" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="40"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="38"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" s="38"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F17" s="8" t="s">
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" s="10"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19" s="10"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="14" t="s">
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="38"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="38"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+    </row>
+    <row r="27" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="38"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A28" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" s="16" t="s">
+      <c r="B28" s="46"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A24" s="13" t="s">
+      <c r="E28" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="17" t="s">
+      <c r="F28" s="22"/>
+      <c r="G28" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-    </row>
-    <row r="27" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="13"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A28" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="E28" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="F28" s="20"/>
-      <c r="G28" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="H28" s="13"/>
-      <c r="I28" s="13"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A29" s="18"/>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A30" s="18"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A31" s="18"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A32" s="18"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A33" s="18"/>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="18"/>
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="46"/>
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="47"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="46"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="47"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="38"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="46"/>
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="47"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" s="46"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="47"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" s="46"/>
+      <c r="B33" s="46"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="47"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="38"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="46"/>
+      <c r="B34" s="46"/>
+      <c r="C34" s="46"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="44">
@@ -1672,22 +1739,17 @@
     <mergeCell ref="G28:I34"/>
     <mergeCell ref="D28:D34"/>
     <mergeCell ref="E28:F34"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="F19:I19"/>
     <mergeCell ref="A20:E22"/>
     <mergeCell ref="F20:I22"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
     <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="D16:I16"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
     <mergeCell ref="F14:I14"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A7:E7"/>
@@ -1697,6 +1759,11 @@
     <mergeCell ref="A11:I11"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="F4:I4"/>

</xml_diff>